<commit_message>
Added order to data
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oneomnicom-my.sharepoint.com/personal/gavin_ransom_omc_com/Documents/Documents/Power Bi/git-demo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{8BFCD240-D87B-4163-8272-CFBE7205E988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{158F87D6-D597-4187-BA3E-81328A7D1C46}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{8BFCD240-D87B-4163-8272-CFBE7205E988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66701861-324B-452E-B333-4B6AF1D43CEC}"/>
   <bookViews>
     <workbookView xWindow="4395" yWindow="-14460" windowWidth="17280" windowHeight="9960" xr2:uid="{8E8DF278-499C-4C14-9881-230D734CF08D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>a</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>dec</t>
+  </si>
+  <si>
+    <t>order</t>
   </si>
 </sst>
 </file>
@@ -449,111 +452,150 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CB79394-C2A6-4977-99FC-71073F8E8833}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
         <v>32</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7">
         <v>26</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10">
         <v>30</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
       <c r="B11">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
       <c r="B12">
         <v>27</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13">
         <v>28</v>
+      </c>
+      <c r="C13">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>